<commit_message>
Add ICML 2026 publication
</commit_message>
<xml_diff>
--- a/publications.xlsx
+++ b/publications.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1069,6 +1069,35 @@
           <t>https://github.com/wuwuz/Vacuum-Filter</t>
         </is>
       </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Continual Learning With Participation Privacy: An Auditable Buffering-Aggregation Recipe</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://openreview.net/forum?id=XfmTSEvETM</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>T-H. Hubert Chan, Elaine Shi, Mengshi Zhao, Mingxun Zhou</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>